<commit_message>
Results cost breakdown 2
</commit_message>
<xml_diff>
--- a/dataCaseStudy_Cement/raw_results/oxy_only/Summary.xlsx
+++ b/dataCaseStudy_Cement/raw_results/oxy_only/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE4"/>
+  <dimension ref="A1:AE7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -891,6 +891,315 @@
       <c r="AE4" t="inlineStr">
         <is>
           <t>dataCaseStudy_Cement\raw_results\oxy_only\20260401174950_carbon_tax_250_el_price_107</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>71309833.48977743</v>
+      </c>
+      <c r="B5" t="n">
+        <v>14288980.05949447</v>
+      </c>
+      <c r="C5" t="n">
+        <v>5951746.54475859</v>
+      </c>
+      <c r="D5" t="n">
+        <v>9370697.908208225</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>23659677.9677027</v>
+      </c>
+      <c r="G5" t="n">
+        <v>5951746.54475859</v>
+      </c>
+      <c r="H5" t="n">
+        <v>32490772.9957337</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>9207635.98158244</v>
+      </c>
+      <c r="M5" t="n">
+        <v>71309833.48977743</v>
+      </c>
+      <c r="N5" t="n">
+        <v>61391.06622803007</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>61391.06622803007</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>61384.23987721677</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" t="n">
+        <v>6.826350813931858</v>
+      </c>
+      <c r="V5" t="n">
+        <v>2.361999988555908</v>
+      </c>
+      <c r="W5" t="n">
+        <v>71309833.48977071</v>
+      </c>
+      <c r="X5" t="n">
+        <v>71309833.48977743</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>6.720423698425293e-06</v>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_107</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\oxy_only\20260401183715_carbon_tax_150_el_price_107</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>59161675.96459493</v>
+      </c>
+      <c r="B6" t="n">
+        <v>17793618.62427595</v>
+      </c>
+      <c r="C6" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D6" t="n">
+        <v>24835293.43733854</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>42628912.0616145</v>
+      </c>
+      <c r="G6" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H6" t="n">
+        <v>9155739.400661327</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>651387.1559713911</v>
+      </c>
+      <c r="M6" t="n">
+        <v>59161675.96459493</v>
+      </c>
+      <c r="N6" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>7237.635066215884</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V6" t="n">
+        <v>2.032000064849854</v>
+      </c>
+      <c r="W6" t="n">
+        <v>59161675.9645758</v>
+      </c>
+      <c r="X6" t="n">
+        <v>59161675.96459493</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>1.913309097290039e-05</v>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>carbon_tax_90_el_price_107</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\oxy_only\20260401183924_carbon_tax_90_el_price_107</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>60319697.57519241</v>
+      </c>
+      <c r="B7" t="n">
+        <v>17793618.62427595</v>
+      </c>
+      <c r="C7" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D7" t="n">
+        <v>24835293.43733854</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>42628912.0616145</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H7" t="n">
+        <v>9155739.400661327</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1809408.766568877</v>
+      </c>
+      <c r="M7" t="n">
+        <v>60319697.57519241</v>
+      </c>
+      <c r="N7" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>7245.844635991023</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>7237.635066215884</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V7" t="n">
+        <v>1.88700008392334</v>
+      </c>
+      <c r="W7" t="n">
+        <v>60319697.57512113</v>
+      </c>
+      <c r="X7" t="n">
+        <v>60319697.57519241</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>7.127970457077026e-05</v>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_107</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\oxy_only\20260401184141_carbon_tax_250_el_price_107</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
results oxy only final
</commit_message>
<xml_diff>
--- a/dataCaseStudy_Cement/raw_results/oxy_only/Summary.xlsx
+++ b/dataCaseStudy_Cement/raw_results/oxy_only/Summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="54">
   <si>
     <t>total_npv</t>
   </si>
@@ -167,6 +167,15 @@
   </si>
   <si>
     <t>dataCaseStudy_Cement\raw_results\oxy_only\20260403164700_carbon_tax_250_el_price_107</t>
+  </si>
+  <si>
+    <t>dataCaseStudy_Cement\raw_results\oxy_only\20260407231558_carbon_tax_150_el_price_107</t>
+  </si>
+  <si>
+    <t>dataCaseStudy_Cement\raw_results\oxy_only\20260407231826_carbon_tax_90_el_price_107</t>
+  </si>
+  <si>
+    <t>dataCaseStudy_Cement\raw_results\oxy_only\20260407232149_carbon_tax_250_el_price_107</t>
   </si>
 </sst>
 </file>
@@ -524,7 +533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE15"/>
+  <dimension ref="A1:AE18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:31">
@@ -1950,6 +1959,291 @@
       </c>
       <c r="AE15" t="s">
         <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:31">
+      <c r="A16">
+        <v>71309833.48977743</v>
+      </c>
+      <c r="B16">
+        <v>14288980.05949447</v>
+      </c>
+      <c r="C16">
+        <v>5951746.54475859</v>
+      </c>
+      <c r="D16">
+        <v>9370697.908208225</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>23659677.9677027</v>
+      </c>
+      <c r="G16">
+        <v>5951746.54475859</v>
+      </c>
+      <c r="H16">
+        <v>32490772.9957337</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>9207635.98158244</v>
+      </c>
+      <c r="M16">
+        <v>71309833.48977743</v>
+      </c>
+      <c r="N16">
+        <v>61391.06622803007</v>
+      </c>
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16">
+        <v>61391.06622803007</v>
+      </c>
+      <c r="Q16">
+        <v>61384.23987721677</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+      <c r="S16">
+        <v>0</v>
+      </c>
+      <c r="T16">
+        <v>0</v>
+      </c>
+      <c r="U16">
+        <v>6.826350813931858</v>
+      </c>
+      <c r="V16">
+        <v>1.36899995803833</v>
+      </c>
+      <c r="W16">
+        <v>71309833.48977071</v>
+      </c>
+      <c r="X16">
+        <v>71309833.48977743</v>
+      </c>
+      <c r="Y16">
+        <v>6.720423698425293E-06</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>31</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB16">
+        <v>0</v>
+      </c>
+      <c r="AC16">
+        <v>1</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE16" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" spans="1:31">
+      <c r="A17">
+        <v>65039542.2226257</v>
+      </c>
+      <c r="B17">
+        <v>13228586.17399643</v>
+      </c>
+      <c r="C17">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="D17">
+        <v>25517441.94529606</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>38746028.1192925</v>
+      </c>
+      <c r="G17">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="H17">
+        <v>7507405.219337072</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>13027743.11917158</v>
+      </c>
+      <c r="M17">
+        <v>65039542.2226257</v>
+      </c>
+      <c r="N17">
+        <v>144759.1919555886</v>
+      </c>
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="P17">
+        <v>144759.1919555886</v>
+      </c>
+      <c r="Q17">
+        <v>144752.7013241411</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+      <c r="S17">
+        <v>0</v>
+      </c>
+      <c r="T17">
+        <v>0</v>
+      </c>
+      <c r="U17">
+        <v>6.49063144699852</v>
+      </c>
+      <c r="V17">
+        <v>3.539000034332275</v>
+      </c>
+      <c r="W17">
+        <v>65039542.22261964</v>
+      </c>
+      <c r="X17">
+        <v>65039542.2226257</v>
+      </c>
+      <c r="Y17">
+        <v>6.057322025299072E-06</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>31</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB17">
+        <v>0</v>
+      </c>
+      <c r="AC17">
+        <v>1</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE17" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:31">
+      <c r="A18">
+        <v>68508980.45020217</v>
+      </c>
+      <c r="B18">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C18">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D18">
+        <v>27323116.73979944</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>44968491.63269403</v>
+      </c>
+      <c r="G18">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H18">
+        <v>15005442.70461023</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>1809408.766550194</v>
+      </c>
+      <c r="M18">
+        <v>68508980.45020217</v>
+      </c>
+      <c r="N18">
+        <v>7245.844635990999</v>
+      </c>
+      <c r="O18">
+        <v>0</v>
+      </c>
+      <c r="P18">
+        <v>7245.844635990999</v>
+      </c>
+      <c r="Q18">
+        <v>7237.635066215867</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+      <c r="S18">
+        <v>0</v>
+      </c>
+      <c r="T18">
+        <v>0</v>
+      </c>
+      <c r="U18">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V18">
+        <v>3.700999975204468</v>
+      </c>
+      <c r="W18">
+        <v>68508980.45018527</v>
+      </c>
+      <c r="X18">
+        <v>68508980.45020217</v>
+      </c>
+      <c r="Y18">
+        <v>1.689791679382324E-05</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>31</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB18">
+        <v>0</v>
+      </c>
+      <c r="AC18">
+        <v>1</v>
+      </c>
+      <c r="AD18" t="s">
+        <v>35</v>
+      </c>
+      <c r="AE18" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
results cost breakdown oxy only
</commit_message>
<xml_diff>
--- a/dataCaseStudy_Cement/raw_results/oxy_only/Summary.xlsx
+++ b/dataCaseStudy_Cement/raw_results/oxy_only/Summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="57">
   <si>
     <t>total_npv</t>
   </si>
@@ -176,6 +176,15 @@
   </si>
   <si>
     <t>dataCaseStudy_Cement\raw_results\oxy_only\20260407232149_carbon_tax_250_el_price_107</t>
+  </si>
+  <si>
+    <t>dataCaseStudy_Cement\raw_results\oxy_only\20260418184440_carbon_tax_150_el_price_107</t>
+  </si>
+  <si>
+    <t>dataCaseStudy_Cement\raw_results\oxy_only\20260418184551_carbon_tax_90_el_price_107</t>
+  </si>
+  <si>
+    <t>dataCaseStudy_Cement\raw_results\oxy_only\20260418184715_carbon_tax_250_el_price_107</t>
   </si>
 </sst>
 </file>
@@ -533,7 +542,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE18"/>
+  <dimension ref="A1:AE21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:31">
@@ -2244,6 +2253,291 @@
       </c>
       <c r="AE18" t="s">
         <v>53</v>
+      </c>
+    </row>
+    <row r="19" spans="1:31">
+      <c r="A19">
+        <v>75652586.69319288</v>
+      </c>
+      <c r="B19">
+        <v>15828554.68961274</v>
+      </c>
+      <c r="C19">
+        <v>5951746.54475859</v>
+      </c>
+      <c r="D19">
+        <v>9943373.656615935</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>25771928.34622867</v>
+      </c>
+      <c r="G19">
+        <v>5951746.54475859</v>
+      </c>
+      <c r="H19">
+        <v>34661743.69143192</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>9267168.110773707</v>
+      </c>
+      <c r="M19">
+        <v>75652586.69319288</v>
+      </c>
+      <c r="N19">
+        <v>61787.94212829441</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <v>61787.94212829441</v>
+      </c>
+      <c r="Q19">
+        <v>61781.12073849188</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+      <c r="S19">
+        <v>0</v>
+      </c>
+      <c r="T19">
+        <v>0</v>
+      </c>
+      <c r="U19">
+        <v>6.821389803165919</v>
+      </c>
+      <c r="V19">
+        <v>0.9330000877380371</v>
+      </c>
+      <c r="W19">
+        <v>75652586.69318601</v>
+      </c>
+      <c r="X19">
+        <v>75652586.69319288</v>
+      </c>
+      <c r="Y19">
+        <v>6.86943531036377E-06</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>31</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB19">
+        <v>0</v>
+      </c>
+      <c r="AC19">
+        <v>1</v>
+      </c>
+      <c r="AD19" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE19" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="1:31">
+      <c r="A20">
+        <v>65039542.2226257</v>
+      </c>
+      <c r="B20">
+        <v>13228586.17399643</v>
+      </c>
+      <c r="C20">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="D20">
+        <v>25517441.94529606</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>38746028.1192925</v>
+      </c>
+      <c r="G20">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="H20">
+        <v>7507405.219337072</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>13027743.11917158</v>
+      </c>
+      <c r="M20">
+        <v>65039542.2226257</v>
+      </c>
+      <c r="N20">
+        <v>144759.1919555886</v>
+      </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20">
+        <v>144759.1919555886</v>
+      </c>
+      <c r="Q20">
+        <v>144752.7013241411</v>
+      </c>
+      <c r="R20">
+        <v>0</v>
+      </c>
+      <c r="S20">
+        <v>0</v>
+      </c>
+      <c r="T20">
+        <v>0</v>
+      </c>
+      <c r="U20">
+        <v>6.49063144699852</v>
+      </c>
+      <c r="V20">
+        <v>4.332000017166138</v>
+      </c>
+      <c r="W20">
+        <v>65039542.22261964</v>
+      </c>
+      <c r="X20">
+        <v>65039542.2226257</v>
+      </c>
+      <c r="Y20">
+        <v>6.057322025299072E-06</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>31</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB20">
+        <v>0</v>
+      </c>
+      <c r="AC20">
+        <v>1</v>
+      </c>
+      <c r="AD20" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" spans="1:31">
+      <c r="A21">
+        <v>68508980.45020217</v>
+      </c>
+      <c r="B21">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C21">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D21">
+        <v>27323116.73979944</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>44968491.63269403</v>
+      </c>
+      <c r="G21">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H21">
+        <v>15005442.70461023</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="L21">
+        <v>1809408.766550194</v>
+      </c>
+      <c r="M21">
+        <v>68508980.45020217</v>
+      </c>
+      <c r="N21">
+        <v>7245.844635990999</v>
+      </c>
+      <c r="O21">
+        <v>0</v>
+      </c>
+      <c r="P21">
+        <v>7245.844635990999</v>
+      </c>
+      <c r="Q21">
+        <v>7237.635066215867</v>
+      </c>
+      <c r="R21">
+        <v>0</v>
+      </c>
+      <c r="S21">
+        <v>0</v>
+      </c>
+      <c r="T21">
+        <v>0</v>
+      </c>
+      <c r="U21">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V21">
+        <v>2.532999992370605</v>
+      </c>
+      <c r="W21">
+        <v>68508980.45018527</v>
+      </c>
+      <c r="X21">
+        <v>68508980.45020217</v>
+      </c>
+      <c r="Y21">
+        <v>1.689791679382324E-05</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>31</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB21">
+        <v>0</v>
+      </c>
+      <c r="AC21">
+        <v>1</v>
+      </c>
+      <c r="AD21" t="s">
+        <v>35</v>
+      </c>
+      <c r="AE21" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
results cement cost breakdown and tech selection
</commit_message>
<xml_diff>
--- a/dataCaseStudy_Cement/raw_results/oxy_only/Summary.xlsx
+++ b/dataCaseStudy_Cement/raw_results/oxy_only/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE25"/>
+  <dimension ref="A1:AE28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3054,6 +3054,315 @@
       <c r="AE25" t="inlineStr">
         <is>
           <t>dataCaseStudy_Cement\raw_results\oxy_only\20260424174332_carbon_tax_250_el_price_107</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>75652586.69319288</v>
+      </c>
+      <c r="B26" t="n">
+        <v>15828554.68961274</v>
+      </c>
+      <c r="C26" t="n">
+        <v>5951746.54475859</v>
+      </c>
+      <c r="D26" t="n">
+        <v>9943373.656615935</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>25771928.34622867</v>
+      </c>
+      <c r="G26" t="n">
+        <v>5951746.54475859</v>
+      </c>
+      <c r="H26" t="n">
+        <v>34661743.69143192</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="n">
+        <v>9267168.110773707</v>
+      </c>
+      <c r="M26" t="n">
+        <v>75652586.69319288</v>
+      </c>
+      <c r="N26" t="n">
+        <v>61787.94212829441</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="n">
+        <v>61787.94212829441</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>61781.12073849188</v>
+      </c>
+      <c r="R26" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" t="n">
+        <v>0</v>
+      </c>
+      <c r="T26" t="n">
+        <v>0</v>
+      </c>
+      <c r="U26" t="n">
+        <v>6.821389803165919</v>
+      </c>
+      <c r="V26" t="n">
+        <v>2.558000087738037</v>
+      </c>
+      <c r="W26" t="n">
+        <v>75652586.69318601</v>
+      </c>
+      <c r="X26" t="n">
+        <v>75652586.69319288</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>6.86943531036377e-06</v>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>carbon_tax_150_el_price_107</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\oxy_only\20260427220430_carbon_tax_150_el_price_107</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>63199832.30501079</v>
+      </c>
+      <c r="B27" t="n">
+        <v>13228586.17399643</v>
+      </c>
+      <c r="C27" t="n">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="D27" t="n">
+        <v>23677732.02768116</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>36906318.20167759</v>
+      </c>
+      <c r="G27" t="n">
+        <v>5758365.764824538</v>
+      </c>
+      <c r="H27" t="n">
+        <v>7507405.219337074</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>13027743.11917158</v>
+      </c>
+      <c r="M27" t="n">
+        <v>63199832.30501079</v>
+      </c>
+      <c r="N27" t="n">
+        <v>144759.1919555883</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>144759.1919555883</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>144752.701324141</v>
+      </c>
+      <c r="R27" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" t="n">
+        <v>0</v>
+      </c>
+      <c r="T27" t="n">
+        <v>0</v>
+      </c>
+      <c r="U27" t="n">
+        <v>6.490631446998519</v>
+      </c>
+      <c r="V27" t="n">
+        <v>3.454999923706055</v>
+      </c>
+      <c r="W27" t="n">
+        <v>63199832.30500505</v>
+      </c>
+      <c r="X27" t="n">
+        <v>63199832.30501079</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>5.736947059631348e-06</v>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>carbon_tax_90_el_price_107</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\oxy_only\20260427220711_carbon_tax_90_el_price_107</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>68855760.08608824</v>
+      </c>
+      <c r="B28" t="n">
+        <v>17645374.89289459</v>
+      </c>
+      <c r="C28" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="D28" t="n">
+        <v>27669896.3756855</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>45315271.26858009</v>
+      </c>
+      <c r="G28" t="n">
+        <v>6725637.346347709</v>
+      </c>
+      <c r="H28" t="n">
+        <v>15005442.70461023</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" t="n">
+        <v>1809408.7665502</v>
+      </c>
+      <c r="M28" t="n">
+        <v>68855760.08608824</v>
+      </c>
+      <c r="N28" t="n">
+        <v>7245.844635990998</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
+        <v>7245.844635990998</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>7237.635066215867</v>
+      </c>
+      <c r="R28" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" t="n">
+        <v>0</v>
+      </c>
+      <c r="U28" t="n">
+        <v>8.209569775222583</v>
+      </c>
+      <c r="V28" t="n">
+        <v>3.913999795913696</v>
+      </c>
+      <c r="W28" t="n">
+        <v>68855760.08607104</v>
+      </c>
+      <c r="X28" t="n">
+        <v>68855760.08608824</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>1.71959400177002e-05</v>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>carbon_tax_250_el_price_107</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\oxy_only\20260427220954_carbon_tax_250_el_price_107</t>
         </is>
       </c>
     </row>

</xml_diff>